<commit_message>
Added all Factions to the model. Added all defined units. Added all defined formations. Added all Historical commanders. Added all defined generic commanders. Made up some new commanders. Found missing formation files and documented. Added prefix to all Faction units.
</commit_message>
<xml_diff>
--- a/assets/ESR Formations-England.xlsx
+++ b/assets/ESR Formations-England.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9efa18f7c2e81ea4/Documents/NewRecruit/ESR_NewRecruit/assets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9EFA18F7C2E81EA4/Documents/NewRecruit/ESR/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="8_{1387204D-2BDB-4948-B700-406CBBECFE5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46C70088-6333-40EF-8DEE-AC9FBA4FD574}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="8_{1387204D-2BDB-4948-B700-406CBBECFE5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACE83BF9-4B19-4FC7-A510-64189CA66F2F}"/>
   <bookViews>
-    <workbookView xWindow="1935" yWindow="525" windowWidth="26610" windowHeight="14700" xr2:uid="{20271C60-C4FB-4B77-A1B3-909BAACA5FD5}"/>
+    <workbookView xWindow="660" yWindow="240" windowWidth="26610" windowHeight="14595" activeTab="1" xr2:uid="{20271C60-C4FB-4B77-A1B3-909BAACA5FD5}"/>
   </bookViews>
   <sheets>
     <sheet name="BaselineFormations" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="55">
   <si>
     <t>Formation</t>
   </si>
@@ -124,18 +124,9 @@
     <t>x</t>
   </si>
   <si>
-    <t>Brigade</t>
-  </si>
-  <si>
     <t>Foot Infantry Battalions</t>
   </si>
   <si>
-    <t>Infantry Division</t>
-  </si>
-  <si>
-    <t>1st Division</t>
-  </si>
-  <si>
     <t>Foot Guards Battalions</t>
   </si>
   <si>
@@ -145,9 +136,6 @@
     <t>Limit one 1st Division</t>
   </si>
   <si>
-    <t>Light Division</t>
-  </si>
-  <si>
     <t>Light Foot Battalions</t>
   </si>
   <si>
@@ -160,21 +148,12 @@
     <t>Limit one Light Division</t>
   </si>
   <si>
-    <t>Light Cavalry Brigade</t>
-  </si>
-  <si>
     <t>Light Dragoon Squadron Groups</t>
   </si>
   <si>
-    <t>[Heavy] Cavalry Brigade</t>
-  </si>
-  <si>
     <t>Dragoon Squadron Groups</t>
   </si>
   <si>
-    <t>Artillery Park</t>
-  </si>
-  <si>
     <t>9-pdr Royal Artillery Battery</t>
   </si>
   <si>
@@ -182,10 +161,6 @@
   </si>
   <si>
     <t>6-pdr Royal Horse Artillery Battery</t>
-  </si>
-  <si>
-    <t>Impetuous
-Rapid Deployment</t>
   </si>
   <si>
     <r>
@@ -213,49 +188,78 @@
     <t>Infantry Company</t>
   </si>
   <si>
-    <t>Foot Guards BR</t>
-  </si>
-  <si>
-    <t>Life Guards BR</t>
-  </si>
-  <si>
-    <t>Royal Horse Guards BR</t>
-  </si>
-  <si>
-    <t>Light Infantry BR</t>
-  </si>
-  <si>
-    <t>Foot Infantry BR</t>
-  </si>
-  <si>
-    <t>Highland Foot Inf BR</t>
-  </si>
-  <si>
-    <t>Fusilier Foot Infantry BR</t>
-  </si>
-  <si>
-    <t>Rifles BR</t>
-  </si>
-  <si>
-    <t>Dragoon Guards BR</t>
-  </si>
-  <si>
-    <t>Dragoons BR</t>
-  </si>
-  <si>
-    <t>Light Dragoons BR</t>
-  </si>
-  <si>
-    <t>Hussars BR</t>
-  </si>
-  <si>
-    <t>9-pdr Royal Artillery BR</t>
-  </si>
-  <si>
-    <t>6-pdr Royal Artillery BR</t>
-  </si>
-  <si>
-    <t>6-pdr Royal Horse Artillery BR</t>
+    <t>BR Foot Guards</t>
+  </si>
+  <si>
+    <t>BR Life Guards</t>
+  </si>
+  <si>
+    <t>BR Royal Horse Guards</t>
+  </si>
+  <si>
+    <t>BR Light Infantry</t>
+  </si>
+  <si>
+    <t>BR Foot Infantry</t>
+  </si>
+  <si>
+    <t>BR Highland Foot Inf</t>
+  </si>
+  <si>
+    <t>BR Fusilier Foot Infantry</t>
+  </si>
+  <si>
+    <t>BR Rifles</t>
+  </si>
+  <si>
+    <t>BR Dragoon Guards</t>
+  </si>
+  <si>
+    <t>BR Dragoons</t>
+  </si>
+  <si>
+    <t>BR Light Dragoons</t>
+  </si>
+  <si>
+    <t>BR Hussars</t>
+  </si>
+  <si>
+    <t>BR 9-pdr Royal Artillery</t>
+  </si>
+  <si>
+    <t>BR 6-pdr Royal Artillery</t>
+  </si>
+  <si>
+    <t>BR 6-pdr Royal Horse Artillery</t>
+  </si>
+  <si>
+    <t>BR Brigade</t>
+  </si>
+  <si>
+    <t>BR Infantry Division</t>
+  </si>
+  <si>
+    <t>BR 1st Division</t>
+  </si>
+  <si>
+    <t>BR Light Division</t>
+  </si>
+  <si>
+    <t>BR Light Cavalry Brigade</t>
+  </si>
+  <si>
+    <t>BR Heavy Cavalry Brigade</t>
+  </si>
+  <si>
+    <t>BR Artillery Park</t>
+  </si>
+  <si>
+    <t>Impetuous,
+Rapid Deployment</t>
+  </si>
+  <si>
+    <t>Impetuous, 
+Rapid Deployment</t>
   </si>
 </sst>
 </file>
@@ -733,21 +737,21 @@
         <v>5</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="57" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E2" s="3">
         <v>3</v>
@@ -757,19 +761,19 @@
     </row>
     <row r="3" spans="1:10" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E3" s="3">
         <v>5</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>10</v>
@@ -777,22 +781,22 @@
     </row>
     <row r="4" spans="1:10" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E4" s="3">
         <v>2</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>11</v>
@@ -800,13 +804,13 @@
     </row>
     <row r="5" spans="1:10" ht="85.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D5" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E5" s="3">
         <v>2</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>11</v>
@@ -814,13 +818,13 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D6" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E6" s="3">
         <v>2</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>10</v>
@@ -828,22 +832,22 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E7" s="3">
         <v>2</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>10</v>
@@ -851,13 +855,13 @@
     </row>
     <row r="8" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D8" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E8" s="3">
         <v>8</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>10</v>
@@ -865,13 +869,13 @@
     </row>
     <row r="9" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D9" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E9" s="3">
         <v>1</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>10</v>
@@ -879,45 +883,45 @@
     </row>
     <row r="10" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="E10" s="3">
         <v>2</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="E11" s="3">
         <v>4</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>11</v>
@@ -925,7 +929,7 @@
     </row>
     <row r="12" spans="1:10" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I12" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>11</v>
@@ -933,7 +937,7 @@
     </row>
     <row r="13" spans="1:10" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>8</v>
@@ -942,13 +946,13 @@
         <v>9</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E13" s="3">
         <v>1</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>11</v>
@@ -956,13 +960,13 @@
     </row>
     <row r="14" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D14" s="3" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="E14" s="3">
         <v>1</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>11</v>
@@ -970,13 +974,13 @@
     </row>
     <row r="15" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D15" s="3" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="E15" s="3">
         <v>1</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>12</v>
@@ -984,7 +988,7 @@
     </row>
     <row r="16" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I16" s="2" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>12</v>
@@ -992,7 +996,7 @@
     </row>
     <row r="17" spans="9:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I17" s="2" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>12</v>
@@ -1028,55 +1032,55 @@
       </c>
       <c r="D1" s="3" t="str" cm="1">
         <f t="array" ref="D1:R1">TRANSPOSE( BaselineFormations!I3:I17 )</f>
-        <v>Foot Guards BR</v>
+        <v>BR Foot Guards</v>
       </c>
       <c r="E1" s="3" t="str">
-        <v>Life Guards BR</v>
+        <v>BR Life Guards</v>
       </c>
       <c r="F1" s="3" t="str">
-        <v>Royal Horse Guards BR</v>
+        <v>BR Royal Horse Guards</v>
       </c>
       <c r="G1" s="3" t="str">
-        <v>Light Infantry BR</v>
+        <v>BR Light Infantry</v>
       </c>
       <c r="H1" s="3" t="str">
-        <v>Foot Infantry BR</v>
+        <v>BR Foot Infantry</v>
       </c>
       <c r="I1" s="3" t="str">
-        <v>Highland Foot Inf BR</v>
+        <v>BR Highland Foot Inf</v>
       </c>
       <c r="J1" s="3" t="str">
-        <v>Fusilier Foot Infantry BR</v>
+        <v>BR Fusilier Foot Infantry</v>
       </c>
       <c r="K1" s="3" t="str">
-        <v>Rifles BR</v>
+        <v>BR Rifles</v>
       </c>
       <c r="L1" s="3" t="str">
-        <v>Dragoon Guards BR</v>
+        <v>BR Dragoon Guards</v>
       </c>
       <c r="M1" s="3" t="str">
-        <v>Dragoons BR</v>
+        <v>BR Dragoons</v>
       </c>
       <c r="N1" s="3" t="str">
-        <v>Light Dragoons BR</v>
+        <v>BR Light Dragoons</v>
       </c>
       <c r="O1" s="3" t="str">
-        <v>Hussars BR</v>
+        <v>BR Hussars</v>
       </c>
       <c r="P1" s="3" t="str">
-        <v>9-pdr Royal Artillery BR</v>
+        <v>BR 9-pdr Royal Artillery</v>
       </c>
       <c r="Q1" s="3" t="str">
-        <v>6-pdr Royal Artillery BR</v>
+        <v>BR 6-pdr Royal Artillery</v>
       </c>
       <c r="R1" s="3" t="str">
-        <v>6-pdr Royal Horse Artillery BR</v>
+        <v>BR 6-pdr Royal Horse Artillery</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="str" cm="1">
         <f t="array" ref="A2:C8">_xlfn.LET(_xlpm.data,_xlfn._xlws.FILTER(BaselineFormations!A:C,(BaselineFormations!A:A&lt;&gt;"Formation")*(NOT(ISBLANK(BaselineFormations!A:A)))),IF(_xlpm.data=0,"",_xlpm.data))</f>
-        <v>Brigade</v>
+        <v>BR Brigade</v>
       </c>
       <c r="B2" t="str">
         <v>Infantry</v>
@@ -1087,10 +1091,22 @@
       <c r="H2" t="s">
         <v>14</v>
       </c>
+      <c r="K2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P2" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
-        <v>Infantry Division</v>
+        <v>BR Infantry Division</v>
       </c>
       <c r="B3" t="str">
         <v>Infantry</v>
@@ -1101,16 +1117,22 @@
       <c r="H3" t="s">
         <v>14</v>
       </c>
+      <c r="K3" t="s">
+        <v>14</v>
+      </c>
       <c r="P3" t="s">
         <v>14</v>
       </c>
       <c r="Q3" t="s">
+        <v>14</v>
+      </c>
+      <c r="R3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
-        <v>1st Division</v>
+        <v>BR 1st Division</v>
       </c>
       <c r="B4" t="str">
         <v>Infantry</v>
@@ -1130,16 +1152,22 @@
       <c r="I4" t="s">
         <v>14</v>
       </c>
+      <c r="K4" t="s">
+        <v>14</v>
+      </c>
       <c r="P4" t="s">
         <v>14</v>
       </c>
       <c r="Q4" t="s">
+        <v>14</v>
+      </c>
+      <c r="R4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
-        <v>Light Division</v>
+        <v>BR Light Division</v>
       </c>
       <c r="B5" t="str">
         <v>Infantry</v>
@@ -1165,13 +1193,13 @@
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
-        <v>Light Cavalry Brigade</v>
+        <v>BR Light Cavalry Brigade</v>
       </c>
       <c r="B6" t="str">
         <v>Cavalry</v>
       </c>
       <c r="C6" t="str">
-        <v>Impetuous
+        <v>Impetuous, 
 Rapid Deployment</v>
       </c>
       <c r="N6" t="s">
@@ -1183,13 +1211,13 @@
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
-        <v>[Heavy] Cavalry Brigade</v>
+        <v>BR Heavy Cavalry Brigade</v>
       </c>
       <c r="B7" t="str">
         <v>Cavalry</v>
       </c>
       <c r="C7" t="str">
-        <v>Impetuous
+        <v>Impetuous,
 Rapid Deployment</v>
       </c>
       <c r="M7" t="s">
@@ -1201,7 +1229,7 @@
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
-        <v>Artillery Park</v>
+        <v>BR Artillery Park</v>
       </c>
       <c r="B8" t="str">
         <v>Artillery</v>

</xml_diff>